<commit_message>
Import optional Active flags from Excel codebooks
</commit_message>
<xml_diff>
--- a/demo/datasets/ai-scribe/codebook.xlsx
+++ b/demo/datasets/ai-scribe/codebook.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -54,9 +49,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -292,7 +286,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -301,13 +295,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -341,17 +335,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -406,8 +389,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -417,7 +398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -426,6 +407,7 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,6 +441,11 @@
           <t>Exclude</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -483,6 +470,11 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,6 +507,11 @@
           <t>Time spent correcting drafts belongs in Workload and time. Missing social context belongs here only when described as an error or omission.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -547,6 +544,11 @@
           <t>Moving drafts into the health record belongs in Fit with the health record.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -575,6 +577,11 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -599,6 +606,11 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -627,6 +639,11 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -655,6 +672,11 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -683,6 +705,11 @@
           <t>Patients' own views of the tool belong under Patient perspectives.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -707,6 +734,11 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -735,6 +767,11 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -759,6 +796,11 @@
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -787,6 +829,11 @@
           <t>Individual patients' reactions to being recorded belong in Consent and comfort.</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -811,6 +858,11 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -835,6 +887,11 @@
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -859,8 +916,13 @@
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>